<commit_message>
fix: update gitignore and remove temp excel files
</commit_message>
<xml_diff>
--- a/resources/test-data/SHARE_MATRIX/data_extracted.xlsx
+++ b/resources/test-data/SHARE_MATRIX/data_extracted.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BSDC\DataComparisonFramework\src\test\resources\test-data\SHARE_MATRIX\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BSDC\DataComparisonFramework_Python\resources\test-data\SHARE_MATRIX\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1073,7 +1073,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1100,6 +1100,8 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1385,8 +1387,11 @@
   <cols>
     <col min="2" max="2" width="29.109375" customWidth="1"/>
     <col min="7" max="7" width="12.88671875" style="6"/>
+    <col min="9" max="9" width="15.21875" customWidth="1"/>
     <col min="21" max="23" width="12.88671875" style="1"/>
-    <col min="32" max="47" width="12.88671875" style="1"/>
+    <col min="32" max="32" width="12.88671875" style="1"/>
+    <col min="33" max="33" width="12.88671875" style="15"/>
+    <col min="34" max="47" width="12.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:57" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -1486,7 +1491,7 @@
       <c r="AF1" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="AG1" s="9" t="s">
+      <c r="AG1" s="8" t="s">
         <v>298</v>
       </c>
       <c r="AH1" s="9" t="s">
@@ -1650,7 +1655,7 @@
       <c r="AF2" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="AG2" s="10" t="s">
+      <c r="AG2" s="14" t="s">
         <v>226</v>
       </c>
       <c r="AH2" s="1" t="s">
@@ -1811,7 +1816,7 @@
       <c r="AF3" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG3" s="1" t="s">
+      <c r="AG3" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH3" s="1" t="s">
@@ -1972,7 +1977,7 @@
       <c r="AF4" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="AG4" s="10" t="s">
+      <c r="AG4" s="14" t="s">
         <v>228</v>
       </c>
       <c r="AH4" s="10" t="s">
@@ -2130,7 +2135,7 @@
       <c r="AF5" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG5" s="1" t="s">
+      <c r="AG5" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH5" s="1" t="s">
@@ -2288,7 +2293,7 @@
       <c r="AF6" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG6" s="1" t="s">
+      <c r="AG6" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH6" s="1" t="s">
@@ -2449,7 +2454,7 @@
       <c r="AF7" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AG7" s="1" t="s">
+      <c r="AG7" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH7" s="1" t="s">
@@ -2607,7 +2612,7 @@
       <c r="AF8" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG8" s="1" t="s">
+      <c r="AG8" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH8" s="1" t="s">
@@ -2765,7 +2770,7 @@
       <c r="AF9" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG9" s="1" t="s">
+      <c r="AG9" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH9" s="1" t="s">
@@ -2923,7 +2928,7 @@
       <c r="AF10" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG10" s="1" t="s">
+      <c r="AG10" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH10" s="1" t="s">
@@ -3081,7 +3086,7 @@
       <c r="AF11" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG11" s="1" t="s">
+      <c r="AG11" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH11" s="1" t="s">
@@ -3239,7 +3244,7 @@
       <c r="AF12" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG12" s="1" t="s">
+      <c r="AG12" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH12" s="1" t="s">
@@ -3397,7 +3402,7 @@
       <c r="AF13" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG13" s="1" t="s">
+      <c r="AG13" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH13" s="1" t="s">
@@ -3555,7 +3560,7 @@
       <c r="AF14" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG14" s="1" t="s">
+      <c r="AG14" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH14" s="1" t="s">
@@ -3713,7 +3718,7 @@
       <c r="AF15" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG15" s="1" t="s">
+      <c r="AG15" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH15" s="1" t="s">
@@ -3871,7 +3876,7 @@
       <c r="AF16" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="AG16" s="1" t="s">
+      <c r="AG16" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH16" s="1" t="s">
@@ -4029,7 +4034,7 @@
       <c r="AF17" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG17" s="1" t="s">
+      <c r="AG17" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH17" s="1" t="s">
@@ -4187,7 +4192,7 @@
       <c r="AF18" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG18" s="1" t="s">
+      <c r="AG18" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH18" s="1" t="s">
@@ -4345,7 +4350,7 @@
       <c r="AF19" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG19" s="1" t="s">
+      <c r="AG19" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH19" s="1" t="s">
@@ -4503,7 +4508,7 @@
       <c r="AF20" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG20" s="1" t="s">
+      <c r="AG20" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH20" s="1" t="s">
@@ -4661,7 +4666,7 @@
       <c r="AF21" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG21" s="1" t="s">
+      <c r="AG21" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH21" s="1" t="s">
@@ -4819,7 +4824,7 @@
       <c r="AF22" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG22" s="1" t="s">
+      <c r="AG22" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH22" s="1" t="s">
@@ -4977,7 +4982,7 @@
       <c r="AF23" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG23" s="1" t="s">
+      <c r="AG23" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH23" s="1" t="s">
@@ -5135,7 +5140,7 @@
       <c r="AF24" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG24" s="1" t="s">
+      <c r="AG24" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH24" s="1" t="s">
@@ -5293,7 +5298,7 @@
       <c r="AF25" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG25" s="1" t="s">
+      <c r="AG25" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH25" s="1" t="s">
@@ -5451,7 +5456,7 @@
       <c r="AF26" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG26" s="1" t="s">
+      <c r="AG26" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH26" s="1" t="s">
@@ -5609,7 +5614,7 @@
       <c r="AF27" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG27" s="1" t="s">
+      <c r="AG27" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH27" s="1" t="s">
@@ -5767,7 +5772,7 @@
       <c r="AF28" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AG28" s="1" t="s">
+      <c r="AG28" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH28" s="1" t="s">
@@ -5925,7 +5930,7 @@
       <c r="AF29" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AG29" s="1" t="s">
+      <c r="AG29" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH29" s="1" t="s">
@@ -6083,7 +6088,7 @@
       <c r="AF30" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AG30" s="1" t="s">
+      <c r="AG30" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH30" s="1" t="s">
@@ -6241,7 +6246,7 @@
       <c r="AF31" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="AG31" s="1" t="s">
+      <c r="AG31" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH31" s="1" t="s">
@@ -6396,7 +6401,7 @@
       <c r="AF32" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AG32" s="1" t="s">
+      <c r="AG32" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH32" s="1" t="s">
@@ -6551,7 +6556,7 @@
       <c r="AF33" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AG33" s="1" t="s">
+      <c r="AG33" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH33" s="1" t="s">
@@ -6706,7 +6711,7 @@
       <c r="AF34" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AG34" s="1" t="s">
+      <c r="AG34" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH34" s="1" t="s">
@@ -6861,7 +6866,7 @@
       <c r="AF35" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AG35" s="1" t="s">
+      <c r="AG35" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH35" s="1" t="s">
@@ -7016,7 +7021,7 @@
       <c r="AF36" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="AG36" s="1" t="s">
+      <c r="AG36" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH36" s="1" t="s">
@@ -7171,7 +7176,7 @@
       <c r="AF37" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="AG37" s="1" t="s">
+      <c r="AG37" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH37" s="1" t="s">
@@ -7326,7 +7331,7 @@
       <c r="AF38" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="AG38" s="1" t="s">
+      <c r="AG38" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH38" s="1" t="s">
@@ -7481,7 +7486,7 @@
       <c r="AF39" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="AG39" s="1" t="s">
+      <c r="AG39" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH39" s="1" t="s">
@@ -7636,7 +7641,7 @@
       <c r="AF40" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="AG40" s="1" t="s">
+      <c r="AG40" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH40" s="1" t="s">
@@ -7791,7 +7796,7 @@
       <c r="AF41" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="AG41" s="1" t="s">
+      <c r="AG41" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH41" s="1" t="s">
@@ -7946,7 +7951,7 @@
       <c r="AF42" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AG42" s="1" t="s">
+      <c r="AG42" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH42" s="1" t="s">
@@ -8101,7 +8106,7 @@
       <c r="AF43" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="AG43" s="1" t="s">
+      <c r="AG43" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH43" s="1" t="s">
@@ -8256,7 +8261,7 @@
       <c r="AF44" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="AG44" s="1" t="s">
+      <c r="AG44" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH44" s="1" t="s">
@@ -8411,7 +8416,7 @@
       <c r="AF45" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="AG45" s="1" t="s">
+      <c r="AG45" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH45" s="1" t="s">
@@ -8566,7 +8571,7 @@
       <c r="AF46" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="AG46" s="1" t="s">
+      <c r="AG46" s="15" t="s">
         <v>231</v>
       </c>
       <c r="AH46" s="1" t="s">
@@ -8724,7 +8729,7 @@
       <c r="AF47" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG47" s="1" t="s">
+      <c r="AG47" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH47" s="1" t="s">
@@ -8882,7 +8887,7 @@
       <c r="AF48" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG48" s="1" t="s">
+      <c r="AG48" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH48" s="1" t="s">
@@ -9040,7 +9045,7 @@
       <c r="AF49" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG49" s="1" t="s">
+      <c r="AG49" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH49" s="1" t="s">
@@ -9198,7 +9203,7 @@
       <c r="AF50" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG50" s="1" t="s">
+      <c r="AG50" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH50" s="1" t="s">
@@ -9356,7 +9361,7 @@
       <c r="AF51" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG51" s="1" t="s">
+      <c r="AG51" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH51" s="1" t="s">
@@ -9514,7 +9519,7 @@
       <c r="AF52" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG52" s="1" t="s">
+      <c r="AG52" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH52" s="1" t="s">
@@ -9672,7 +9677,7 @@
       <c r="AF53" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG53" s="1" t="s">
+      <c r="AG53" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH53" s="1" t="s">
@@ -9830,7 +9835,7 @@
       <c r="AF54" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG54" s="1" t="s">
+      <c r="AG54" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH54" s="1" t="s">
@@ -9991,7 +9996,7 @@
       <c r="AF55" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG55" s="1" t="s">
+      <c r="AG55" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH55" s="1" t="s">
@@ -10152,7 +10157,7 @@
       <c r="AF56" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG56" s="1" t="s">
+      <c r="AG56" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH56" s="1" t="s">
@@ -10313,7 +10318,7 @@
       <c r="AF57" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG57" s="1" t="s">
+      <c r="AG57" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH57" s="1" t="s">
@@ -10474,7 +10479,7 @@
       <c r="AF58" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG58" s="1" t="s">
+      <c r="AG58" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH58" s="1" t="s">
@@ -10635,7 +10640,7 @@
       <c r="AF59" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG59" s="1" t="s">
+      <c r="AG59" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH59" s="1" t="s">
@@ -10796,7 +10801,7 @@
       <c r="AF60" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG60" s="1" t="s">
+      <c r="AG60" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH60" s="1" t="s">
@@ -10957,7 +10962,7 @@
       <c r="AF61" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG61" s="1" t="s">
+      <c r="AG61" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH61" s="1" t="s">
@@ -11118,7 +11123,7 @@
       <c r="AF62" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG62" s="1" t="s">
+      <c r="AG62" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH62" s="1" t="s">
@@ -11279,7 +11284,7 @@
       <c r="AF63" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG63" s="1" t="s">
+      <c r="AG63" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH63" s="1" t="s">
@@ -11440,7 +11445,7 @@
       <c r="AF64" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG64" s="1" t="s">
+      <c r="AG64" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH64" s="1" t="s">
@@ -11601,7 +11606,7 @@
       <c r="AF65" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AG65" s="1" t="s">
+      <c r="AG65" s="15" t="s">
         <v>228</v>
       </c>
       <c r="AH65" s="1" t="s">
@@ -11759,7 +11764,7 @@
       <c r="AF66" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG66" s="1" t="s">
+      <c r="AG66" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH66" s="1" t="s">
@@ -11917,7 +11922,7 @@
       <c r="AF67" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG67" s="1" t="s">
+      <c r="AG67" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH67" s="1" t="s">
@@ -12075,7 +12080,7 @@
       <c r="AF68" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG68" s="1" t="s">
+      <c r="AG68" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH68" s="1" t="s">
@@ -12233,7 +12238,7 @@
       <c r="AF69" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG69" s="1" t="s">
+      <c r="AG69" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH69" s="1" t="s">
@@ -12391,7 +12396,7 @@
       <c r="AF70" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG70" s="1" t="s">
+      <c r="AG70" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH70" s="1" t="s">
@@ -12549,7 +12554,7 @@
       <c r="AF71" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG71" s="1" t="s">
+      <c r="AG71" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH71" s="1" t="s">
@@ -12707,7 +12712,7 @@
       <c r="AF72" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG72" s="1" t="s">
+      <c r="AG72" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH72" s="1" t="s">
@@ -12865,7 +12870,7 @@
       <c r="AF73" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG73" s="1" t="s">
+      <c r="AG73" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH73" s="1" t="s">
@@ -13023,7 +13028,7 @@
       <c r="AF74" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG74" s="1" t="s">
+      <c r="AG74" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH74" s="1" t="s">
@@ -13181,7 +13186,7 @@
       <c r="AF75" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG75" s="1" t="s">
+      <c r="AG75" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH75" s="1" t="s">
@@ -13339,7 +13344,7 @@
       <c r="AF76" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG76" s="1" t="s">
+      <c r="AG76" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH76" s="1" t="s">
@@ -13497,7 +13502,7 @@
       <c r="AF77" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG77" s="1" t="s">
+      <c r="AG77" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH77" s="1" t="s">
@@ -13655,7 +13660,7 @@
       <c r="AF78" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG78" s="1" t="s">
+      <c r="AG78" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH78" s="1" t="s">
@@ -13813,7 +13818,7 @@
       <c r="AF79" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG79" s="1" t="s">
+      <c r="AG79" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH79" s="1" t="s">
@@ -13971,7 +13976,7 @@
       <c r="AF80" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG80" s="1" t="s">
+      <c r="AG80" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH80" s="1" t="s">
@@ -14129,7 +14134,7 @@
       <c r="AF81" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG81" s="1" t="s">
+      <c r="AG81" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH81" s="1" t="s">
@@ -14287,7 +14292,7 @@
       <c r="AF82" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG82" s="1" t="s">
+      <c r="AG82" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH82" s="1" t="s">
@@ -14445,7 +14450,7 @@
       <c r="AF83" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG83" s="1" t="s">
+      <c r="AG83" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH83" s="1" t="s">
@@ -14603,7 +14608,7 @@
       <c r="AF84" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG84" s="1" t="s">
+      <c r="AG84" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH84" s="1" t="s">
@@ -14761,7 +14766,7 @@
       <c r="AF85" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG85" s="1" t="s">
+      <c r="AG85" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH85" s="1" t="s">
@@ -14919,7 +14924,7 @@
       <c r="AF86" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG86" s="1" t="s">
+      <c r="AG86" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH86" s="1" t="s">
@@ -15077,7 +15082,7 @@
       <c r="AF87" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG87" s="1" t="s">
+      <c r="AG87" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH87" s="1" t="s">
@@ -15235,7 +15240,7 @@
       <c r="AF88" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG88" s="1" t="s">
+      <c r="AG88" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH88" s="1" t="s">
@@ -15393,7 +15398,7 @@
       <c r="AF89" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG89" s="1" t="s">
+      <c r="AG89" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH89" s="1" t="s">
@@ -15551,7 +15556,7 @@
       <c r="AF90" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG90" s="1" t="s">
+      <c r="AG90" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH90" s="1" t="s">
@@ -15709,7 +15714,7 @@
       <c r="AF91" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG91" s="1" t="s">
+      <c r="AG91" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH91" s="1" t="s">
@@ -15867,7 +15872,7 @@
       <c r="AF92" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG92" s="1" t="s">
+      <c r="AG92" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH92" s="1" t="s">
@@ -16025,7 +16030,7 @@
       <c r="AF93" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG93" s="1" t="s">
+      <c r="AG93" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH93" s="1" t="s">
@@ -16183,7 +16188,7 @@
       <c r="AF94" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG94" s="1" t="s">
+      <c r="AG94" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH94" s="1" t="s">
@@ -16341,7 +16346,7 @@
       <c r="AF95" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG95" s="1" t="s">
+      <c r="AG95" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH95" s="1" t="s">
@@ -16499,7 +16504,7 @@
       <c r="AF96" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG96" s="1" t="s">
+      <c r="AG96" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH96" s="1" t="s">
@@ -16657,7 +16662,7 @@
       <c r="AF97" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG97" s="1" t="s">
+      <c r="AG97" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH97" s="1" t="s">
@@ -16815,7 +16820,7 @@
       <c r="AF98" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG98" s="1" t="s">
+      <c r="AG98" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH98" s="1" t="s">
@@ -16973,7 +16978,7 @@
       <c r="AF99" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG99" s="1" t="s">
+      <c r="AG99" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH99" s="1" t="s">
@@ -17131,7 +17136,7 @@
       <c r="AF100" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG100" s="1" t="s">
+      <c r="AG100" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH100" s="1" t="s">
@@ -17289,7 +17294,7 @@
       <c r="AF101" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG101" s="1" t="s">
+      <c r="AG101" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH101" s="1" t="s">
@@ -17447,7 +17452,7 @@
       <c r="AF102" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG102" s="1" t="s">
+      <c r="AG102" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH102" s="1" t="s">
@@ -17605,7 +17610,7 @@
       <c r="AF103" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG103" s="1" t="s">
+      <c r="AG103" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH103" s="1" t="s">
@@ -17763,7 +17768,7 @@
       <c r="AF104" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG104" s="1" t="s">
+      <c r="AG104" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH104" s="1" t="s">
@@ -17921,7 +17926,7 @@
       <c r="AF105" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG105" s="1" t="s">
+      <c r="AG105" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH105" s="1" t="s">
@@ -18079,7 +18084,7 @@
       <c r="AF106" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG106" s="1" t="s">
+      <c r="AG106" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH106" s="1" t="s">
@@ -18237,7 +18242,7 @@
       <c r="AF107" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG107" s="1" t="s">
+      <c r="AG107" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH107" s="1" t="s">
@@ -18395,7 +18400,7 @@
       <c r="AF108" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG108" s="1" t="s">
+      <c r="AG108" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH108" s="1" t="s">
@@ -18553,7 +18558,7 @@
       <c r="AF109" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG109" s="1" t="s">
+      <c r="AG109" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH109" s="1" t="s">
@@ -18711,7 +18716,7 @@
       <c r="AF110" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG110" s="1" t="s">
+      <c r="AG110" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH110" s="1" t="s">
@@ -18869,7 +18874,7 @@
       <c r="AF111" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG111" s="1" t="s">
+      <c r="AG111" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH111" s="1" t="s">
@@ -19030,7 +19035,7 @@
       <c r="AF112" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG112" s="1" t="s">
+      <c r="AG112" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH112" s="1" t="s">
@@ -19191,7 +19196,7 @@
       <c r="AF113" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG113" s="1" t="s">
+      <c r="AG113" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH113" s="1" t="s">
@@ -19352,7 +19357,7 @@
       <c r="AF114" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG114" s="1" t="s">
+      <c r="AG114" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH114" s="1" t="s">
@@ -19513,7 +19518,7 @@
       <c r="AF115" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG115" s="1" t="s">
+      <c r="AG115" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH115" s="1" t="s">
@@ -19674,7 +19679,7 @@
       <c r="AF116" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG116" s="1" t="s">
+      <c r="AG116" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH116" s="1" t="s">
@@ -19835,7 +19840,7 @@
       <c r="AF117" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG117" s="1" t="s">
+      <c r="AG117" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH117" s="1" t="s">
@@ -19993,7 +19998,7 @@
       <c r="AF118" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG118" s="1" t="s">
+      <c r="AG118" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH118" s="1" t="s">
@@ -20151,7 +20156,7 @@
       <c r="AF119" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG119" s="1" t="s">
+      <c r="AG119" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH119" s="1" t="s">
@@ -20309,7 +20314,7 @@
       <c r="AF120" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG120" s="1" t="s">
+      <c r="AG120" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH120" s="1" t="s">
@@ -20467,7 +20472,7 @@
       <c r="AF121" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG121" s="1" t="s">
+      <c r="AG121" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH121" s="1" t="s">
@@ -20625,7 +20630,7 @@
       <c r="AF122" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG122" s="1" t="s">
+      <c r="AG122" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH122" s="1" t="s">
@@ -20783,7 +20788,7 @@
       <c r="AF123" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG123" s="1" t="s">
+      <c r="AG123" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH123" s="1" t="s">
@@ -20941,7 +20946,7 @@
       <c r="AF124" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG124" s="1" t="s">
+      <c r="AG124" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH124" s="1" t="s">
@@ -21099,7 +21104,7 @@
       <c r="AF125" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG125" s="1" t="s">
+      <c r="AG125" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH125" s="1" t="s">
@@ -21257,7 +21262,7 @@
       <c r="AF126" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG126" s="1" t="s">
+      <c r="AG126" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH126" s="1" t="s">
@@ -21415,7 +21420,7 @@
       <c r="AF127" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG127" s="1" t="s">
+      <c r="AG127" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH127" s="1" t="s">
@@ -21576,7 +21581,7 @@
       <c r="AF128" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG128" s="1" t="s">
+      <c r="AG128" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH128" s="1" t="s">
@@ -21737,7 +21742,7 @@
       <c r="AF129" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG129" s="1" t="s">
+      <c r="AG129" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH129" s="1" t="s">
@@ -21898,7 +21903,7 @@
       <c r="AF130" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG130" s="1" t="s">
+      <c r="AG130" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH130" s="1" t="s">
@@ -22059,7 +22064,7 @@
       <c r="AF131" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG131" s="1" t="s">
+      <c r="AG131" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH131" s="1" t="s">
@@ -22220,7 +22225,7 @@
       <c r="AF132" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG132" s="1" t="s">
+      <c r="AG132" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH132" s="1" t="s">
@@ -22381,7 +22386,7 @@
       <c r="AF133" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG133" s="1" t="s">
+      <c r="AG133" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH133" s="1" t="s">
@@ -22542,7 +22547,7 @@
       <c r="AF134" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG134" s="1" t="s">
+      <c r="AG134" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH134" s="1" t="s">
@@ -22703,7 +22708,7 @@
       <c r="AF135" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG135" s="1" t="s">
+      <c r="AG135" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH135" s="1" t="s">
@@ -22864,7 +22869,7 @@
       <c r="AF136" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG136" s="1" t="s">
+      <c r="AG136" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH136" s="1" t="s">
@@ -23025,7 +23030,7 @@
       <c r="AF137" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG137" s="1" t="s">
+      <c r="AG137" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH137" s="1" t="s">
@@ -23186,7 +23191,7 @@
       <c r="AF138" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG138" s="1" t="s">
+      <c r="AG138" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH138" s="1" t="s">
@@ -23347,7 +23352,7 @@
       <c r="AF139" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG139" s="1" t="s">
+      <c r="AG139" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH139" s="1" t="s">
@@ -23505,7 +23510,7 @@
       <c r="AF140" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG140" s="1" t="s">
+      <c r="AG140" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH140" s="1" t="s">
@@ -23663,7 +23668,7 @@
       <c r="AF141" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG141" s="1" t="s">
+      <c r="AG141" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH141" s="1" t="s">
@@ -23824,7 +23829,7 @@
       <c r="AF142" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG142" s="1" t="s">
+      <c r="AG142" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH142" s="1" t="s">
@@ -23985,7 +23990,7 @@
       <c r="AF143" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG143" s="1" t="s">
+      <c r="AG143" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH143" s="1" t="s">
@@ -24146,7 +24151,7 @@
       <c r="AF144" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="AG144" s="1" t="s">
+      <c r="AG144" s="15" t="s">
         <v>226</v>
       </c>
       <c r="AH144" s="1" t="s">

</xml_diff>